<commit_message>
Petite Cup 42 (S3 R13): justMaki wins again
Jake takes silver, B_ES surprise 3rd, Sterben 4th.
Maki now 8 wins in 12 rounds. Jake closes to 1620 (#2).
Maps by Lexer & Shadynook.
</commit_message>
<xml_diff>
--- a/Petite Cups 41-45.xlsx
+++ b/Petite Cups 41-45.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D35"/>
+  <dimension ref="A2:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -422,6 +422,11 @@
           <t>Petite Cup 41</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Petite Cup 42</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -429,6 +434,11 @@
           <t>Sahara Sunset by OccasionallyAmazingGamer &amp; Test Subject #50836 by AndMe17</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Map: Lexer &amp; Shadynook</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -447,6 +457,26 @@
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -464,6 +494,17 @@
       <c r="C6" t="n">
         <v>24.04606</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>19.34823</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -480,6 +521,20 @@
       <c r="D7" t="n">
         <v>14</v>
       </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[SWMG]JakeAdjacent</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>19.37091</v>
+      </c>
+      <c r="J7" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -496,6 +551,20 @@
       <c r="D8" t="n">
         <v>13</v>
       </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>B_ES</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>23.07547</v>
+      </c>
+      <c r="J8" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -512,6 +581,20 @@
       <c r="D9" t="n">
         <v>12</v>
       </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>19.71206</v>
+      </c>
+      <c r="J9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -528,6 +611,20 @@
       <c r="D10" t="n">
         <v>11</v>
       </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>22.92393</v>
+      </c>
+      <c r="J10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -544,6 +641,20 @@
       <c r="D11" t="n">
         <v>10</v>
       </c>
+      <c r="G11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>19.57869</v>
+      </c>
+      <c r="J11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -560,6 +671,20 @@
       <c r="D12" t="n">
         <v>10</v>
       </c>
+      <c r="G12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>JobW</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>23.22958</v>
+      </c>
+      <c r="J12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -576,6 +701,20 @@
       <c r="D13" t="n">
         <v>9</v>
       </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>23.26644</v>
+      </c>
+      <c r="J13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -592,6 +731,20 @@
       <c r="D14" t="n">
         <v>9</v>
       </c>
+      <c r="G14" t="n">
+        <v>9</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[CSC] redal</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>19.76407</v>
+      </c>
+      <c r="J14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -608,6 +761,20 @@
       <c r="D15" t="n">
         <v>8</v>
       </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>19.87367</v>
+      </c>
+      <c r="J15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -624,6 +791,20 @@
       <c r="D16" t="n">
         <v>8</v>
       </c>
+      <c r="G16" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>23.22771</v>
+      </c>
+      <c r="J16" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -640,6 +821,20 @@
       <c r="D17" t="n">
         <v>7</v>
       </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>23.42572</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -656,6 +851,20 @@
       <c r="D18" t="n">
         <v>7</v>
       </c>
+      <c r="G18" t="n">
+        <v>13</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>[KURK] Quickracer10</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>19.86061</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -672,6 +881,20 @@
       <c r="D19" t="n">
         <v>6</v>
       </c>
+      <c r="G19" t="n">
+        <v>14</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>23.37241</v>
+      </c>
+      <c r="J19" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -688,6 +911,20 @@
       <c r="D20" t="n">
         <v>6</v>
       </c>
+      <c r="G20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>23.42514</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -704,6 +941,20 @@
       <c r="D21" t="n">
         <v>6</v>
       </c>
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>23.5043</v>
+      </c>
+      <c r="J21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -720,6 +971,20 @@
       <c r="D22" t="n">
         <v>5</v>
       </c>
+      <c r="G22" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>cactuzhead</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>23.90089</v>
+      </c>
+      <c r="J22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -736,6 +1001,20 @@
       <c r="D23" t="n">
         <v>5</v>
       </c>
+      <c r="G23" t="n">
+        <v>18</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>[NewB] Zeus</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>20.26912</v>
+      </c>
+      <c r="J23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -754,6 +1033,20 @@
       <c r="D24" t="n">
         <v>5</v>
       </c>
+      <c r="G24" t="n">
+        <v>19</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>20.4171</v>
+      </c>
+      <c r="J24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -770,6 +1063,20 @@
       <c r="D25" t="n">
         <v>4</v>
       </c>
+      <c r="G25" t="n">
+        <v>20</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>20.75734</v>
+      </c>
+      <c r="J25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -788,6 +1095,20 @@
       <c r="D26" t="n">
         <v>4</v>
       </c>
+      <c r="G26" t="n">
+        <v>21</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>koz</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>23.89353</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -806,6 +1127,20 @@
       <c r="D27" t="n">
         <v>4</v>
       </c>
+      <c r="G27" t="n">
+        <v>22</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>24.10065</v>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -824,6 +1159,20 @@
       <c r="D28" t="n">
         <v>3</v>
       </c>
+      <c r="G28" t="n">
+        <v>23</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>[GECK]R0nanC</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>24.14223</v>
+      </c>
+      <c r="J28" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -842,6 +1191,20 @@
       <c r="D29" t="n">
         <v>3</v>
       </c>
+      <c r="G29" t="n">
+        <v>24</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>22.3696</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -860,6 +1223,20 @@
       <c r="D30" t="n">
         <v>3</v>
       </c>
+      <c r="G30" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>MadZitrone</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>22.51462</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -878,6 +1255,20 @@
       <c r="D31" t="n">
         <v>2</v>
       </c>
+      <c r="G31" t="n">
+        <v>26</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>23.16854</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -896,6 +1287,20 @@
       <c r="D32" t="n">
         <v>2</v>
       </c>
+      <c r="G32" t="n">
+        <v>27</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>25.20982</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -914,6 +1319,20 @@
       <c r="D33" t="n">
         <v>2</v>
       </c>
+      <c r="G33" t="n">
+        <v>28</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Fly8oy</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>26.0627</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -932,6 +1351,20 @@
       <c r="D34" t="n">
         <v>2</v>
       </c>
+      <c r="G34" t="n">
+        <v>29</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>[fn]Form</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>20.20107</v>
+      </c>
+      <c r="J34" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -949,6 +1382,52 @@
       </c>
       <c r="D35" t="n">
         <v>2</v>
+      </c>
+      <c r="G35" t="n">
+        <v>30</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>[its] it_is_nic</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>23.69469</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" t="n">
+        <v>31</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>FF_11</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>24.65928</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="G37" t="n">
+        <v>31</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>True Chaotic Neutral</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>23.73474</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Petite Cup 43 (S3 R14): justMaki wins, Jake 2nd again
30 players. Maki 1st (23.530 in final), Jake 2nd (23.678) — third
consecutive petite finals for these two (41, 42, 43). Top 6: Maki,
Jake, ping, Mμ, Victor, Lexer. aizpun 9th place (deepest petite run,
eliminated R8 on time 24.43).
</commit_message>
<xml_diff>
--- a/Petite Cups 41-45.xlsx
+++ b/Petite Cups 41-45.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J37"/>
+  <dimension ref="A2:P37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -427,6 +427,11 @@
           <t>Petite Cup 42</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Petite Cup 43</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -439,6 +444,11 @@
           <t>Map: Lexer &amp; Shadynook</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Map: TBD (see VOD)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -477,6 +487,26 @@
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -505,6 +535,17 @@
       <c r="I6" t="n">
         <v>19.34823</v>
       </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>23.53025</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -535,6 +576,20 @@
       <c r="J7" t="n">
         <v>15</v>
       </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>23.67819</v>
+      </c>
+      <c r="P7" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -565,6 +620,20 @@
       <c r="J8" t="n">
         <v>14</v>
       </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>20.07159</v>
+      </c>
+      <c r="P8" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -595,6 +664,22 @@
       <c r="J9" t="n">
         <v>13</v>
       </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -625,6 +710,20 @@
       <c r="J10" t="n">
         <v>12</v>
       </c>
+      <c r="M10" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>20.13033</v>
+      </c>
+      <c r="P10" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -655,6 +754,20 @@
       <c r="J11" t="n">
         <v>11</v>
       </c>
+      <c r="M11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>24.03749</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -685,6 +798,20 @@
       <c r="J12" t="n">
         <v>10</v>
       </c>
+      <c r="M12" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>20.27931</v>
+      </c>
+      <c r="P12" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -715,6 +842,20 @@
       <c r="J13" t="n">
         <v>10</v>
       </c>
+      <c r="M13" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>20.5414</v>
+      </c>
+      <c r="P13" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -745,6 +886,20 @@
       <c r="J14" t="n">
         <v>9</v>
       </c>
+      <c r="M14" t="n">
+        <v>9</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>24.43473</v>
+      </c>
+      <c r="P14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -775,6 +930,22 @@
       <c r="J15" t="n">
         <v>9</v>
       </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -805,6 +976,20 @@
       <c r="J16" t="n">
         <v>8</v>
       </c>
+      <c r="M16" t="n">
+        <v>11</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>20.3443</v>
+      </c>
+      <c r="P16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -835,6 +1020,22 @@
       <c r="J17" t="n">
         <v>8</v>
       </c>
+      <c r="M17" t="n">
+        <v>12</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -865,6 +1066,20 @@
       <c r="J18" t="n">
         <v>7</v>
       </c>
+      <c r="M18" t="n">
+        <v>13</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>[CSC] OccasionallyAmazingGamer</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>24.78899</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -895,6 +1110,20 @@
       <c r="J19" t="n">
         <v>7</v>
       </c>
+      <c r="M19" t="n">
+        <v>14</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>24.81317</v>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -925,6 +1154,22 @@
       <c r="J20" t="n">
         <v>6</v>
       </c>
+      <c r="M20" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>[MMM]LKat</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -955,6 +1200,20 @@
       <c r="J21" t="n">
         <v>6</v>
       </c>
+      <c r="M21" t="n">
+        <v>16</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>[GECK]R0nanC</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>20.68511</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -985,6 +1244,20 @@
       <c r="J22" t="n">
         <v>6</v>
       </c>
+      <c r="M22" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>20.70262</v>
+      </c>
+      <c r="P22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1015,6 +1288,20 @@
       <c r="J23" t="n">
         <v>5</v>
       </c>
+      <c r="M23" t="n">
+        <v>18</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>[CSC]ShyGirlyRaccoon</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>20.72788</v>
+      </c>
+      <c r="P23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1047,6 +1334,20 @@
       <c r="J24" t="n">
         <v>5</v>
       </c>
+      <c r="M24" t="n">
+        <v>19</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>ElectricCaveman</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>25.92201</v>
+      </c>
+      <c r="P24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1077,6 +1378,20 @@
       <c r="J25" t="n">
         <v>5</v>
       </c>
+      <c r="M25" t="n">
+        <v>20</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>๖ۣۜNamo ツ</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>26.31735</v>
+      </c>
+      <c r="P25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1109,6 +1424,22 @@
       <c r="J26" t="n">
         <v>4</v>
       </c>
+      <c r="M26" t="n">
+        <v>21</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1141,6 +1472,20 @@
       <c r="J27" t="n">
         <v>4</v>
       </c>
+      <c r="M27" t="n">
+        <v>22</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>PewX [.de]</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>21.28175</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1173,6 +1518,20 @@
       <c r="J28" t="n">
         <v>4</v>
       </c>
+      <c r="M28" t="n">
+        <v>23</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Kilandor</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>21.35589</v>
+      </c>
+      <c r="P28" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1205,6 +1564,20 @@
       <c r="J29" t="n">
         <v>3</v>
       </c>
+      <c r="M29" t="n">
+        <v>24</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>FedtStensDyr</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>21.80087</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1237,6 +1610,22 @@
       <c r="J30" t="n">
         <v>3</v>
       </c>
+      <c r="M30" t="n">
+        <v>25</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Spatial</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1269,6 +1658,22 @@
       <c r="J31" t="n">
         <v>3</v>
       </c>
+      <c r="M31" t="n">
+        <v>25</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>[TTR]DragonShadow84290</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1301,6 +1706,22 @@
       <c r="J32" t="n">
         <v>2</v>
       </c>
+      <c r="M32" t="n">
+        <v>25</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>[Tame]stindt</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1333,6 +1754,20 @@
       <c r="J33" t="n">
         <v>2</v>
       </c>
+      <c r="M33" t="n">
+        <v>28</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Articus</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>26.48379</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1365,6 +1800,22 @@
       <c r="J34" t="n">
         <v>2</v>
       </c>
+      <c r="M34" t="n">
+        <v>29</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>[20x]K410K3N</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1395,6 +1846,22 @@
         <v>23.69469</v>
       </c>
       <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>29</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>duff_mans_jnr</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cup 43 fix: icRS had valid time 20.249 in R7 (left mid-cup)
Added parse_petite_log.py — cross-checks COTDTracker log against
LiveLeaderboardLogger mid-round data to detect DNFs that should be
real times. Flags players who set a valid time then left before round
end, and reranks them within the elimination group by time.

Applied to cup 43: icRS (20.249, from leaving mid-R7) swaps with
Eclipse135 (20.3443) — icRS now pos 11, Eclipse pos 12. PCDJ points
unchanged (both outside top-10 scoring) but the result is accurate.

The parser uses time-range filtering per round to reject previous-map
carryover: petite alternates 2 maps and the leaderboard retains times
between rotations. Only overrides where the candidate time falls
within the current round's time range get applied.
</commit_message>
<xml_diff>
--- a/Petite Cups 41-45.xlsx
+++ b/Petite Cups 41-45.xlsx
@@ -981,11 +981,11 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Eclipse135</t>
+          <t>icRS</t>
         </is>
       </c>
       <c r="O16" t="n">
-        <v>20.3443</v>
+        <v>20.249</v>
       </c>
       <c r="P16" t="n">
         <v>7</v>
@@ -1025,13 +1025,11 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>icRS</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>20.3443</v>
       </c>
       <c r="P17" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
PCDJ Cup 44 — justMaki wins on Petite Tropiques Féminins
</commit_message>
<xml_diff>
--- a/Petite Cups 41-45.xlsx
+++ b/Petite Cups 41-45.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:P37"/>
+  <dimension ref="A2:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -432,6 +432,11 @@
           <t>Petite Cup 43</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Petite Cup 44</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -449,6 +454,11 @@
           <t>Map: TBD (see VOD)</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ - Dungeon Descent + PCDJ 44 - Petite Tropiques Féminins</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -507,6 +517,26 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -546,6 +576,17 @@
       <c r="O6" t="n">
         <v>23.53025</v>
       </c>
+      <c r="S6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>24.49382</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -590,6 +631,20 @@
       <c r="P7" t="n">
         <v>14</v>
       </c>
+      <c r="S7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>25.92793</v>
+      </c>
+      <c r="V7" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -634,6 +689,20 @@
       <c r="P8" t="n">
         <v>13</v>
       </c>
+      <c r="S8" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[WASH] ZOMAN</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>23.16791</v>
+      </c>
+      <c r="V8" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -680,6 +749,20 @@
       <c r="P9" t="n">
         <v>12</v>
       </c>
+      <c r="S9" t="n">
+        <v>4</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>24.77693</v>
+      </c>
+      <c r="V9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -724,6 +807,20 @@
       <c r="P10" t="n">
         <v>11</v>
       </c>
+      <c r="S10" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>[KURK] Quickracer10</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>23.19836</v>
+      </c>
+      <c r="V10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -768,6 +865,22 @@
       <c r="P11" t="n">
         <v>10</v>
       </c>
+      <c r="S11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -812,6 +925,20 @@
       <c r="P12" t="n">
         <v>9</v>
       </c>
+      <c r="S12" t="n">
+        <v>7</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>23.31095</v>
+      </c>
+      <c r="V12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -856,6 +983,20 @@
       <c r="P13" t="n">
         <v>9</v>
       </c>
+      <c r="S13" t="n">
+        <v>8</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>23.343</v>
+      </c>
+      <c r="V13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -900,6 +1041,20 @@
       <c r="P14" t="n">
         <v>8</v>
       </c>
+      <c r="S14" t="n">
+        <v>9</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>[ERR]ferinine</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>25.16142</v>
+      </c>
+      <c r="V14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -946,6 +1101,22 @@
       <c r="P15" t="n">
         <v>8</v>
       </c>
+      <c r="S15" t="n">
+        <v>10</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -990,6 +1161,20 @@
       <c r="P16" t="n">
         <v>7</v>
       </c>
+      <c r="S16" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>23.58802</v>
+      </c>
+      <c r="V16" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1219,20 @@
       <c r="P17" t="n">
         <v>7</v>
       </c>
+      <c r="S17" t="n">
+        <v>12</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>23.60028</v>
+      </c>
+      <c r="V17" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1078,6 +1277,20 @@
       <c r="P18" t="n">
         <v>6</v>
       </c>
+      <c r="S18" t="n">
+        <v>13</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>25.90944</v>
+      </c>
+      <c r="V18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1122,6 +1335,22 @@
       <c r="P19" t="n">
         <v>6</v>
       </c>
+      <c r="S19" t="n">
+        <v>14</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1168,6 +1397,20 @@
       <c r="P20" t="n">
         <v>6</v>
       </c>
+      <c r="S20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>23.62606</v>
+      </c>
+      <c r="V20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1212,6 +1455,20 @@
       <c r="P21" t="n">
         <v>5</v>
       </c>
+      <c r="S21" t="n">
+        <v>16</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>[GECK]R0nanC</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>23.65387</v>
+      </c>
+      <c r="V21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1256,6 +1513,22 @@
       <c r="P22" t="n">
         <v>5</v>
       </c>
+      <c r="S22" t="n">
+        <v>17</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Arepuz</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1300,6 +1573,20 @@
       <c r="P23" t="n">
         <v>5</v>
       </c>
+      <c r="S23" t="n">
+        <v>18</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>29.27843</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1346,6 +1633,20 @@
       <c r="P24" t="n">
         <v>4</v>
       </c>
+      <c r="S24" t="n">
+        <v>19</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>29.65201</v>
+      </c>
+      <c r="V24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1390,6 +1691,22 @@
       <c r="P25" t="n">
         <v>4</v>
       </c>
+      <c r="S25" t="n">
+        <v>20</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1438,6 +1755,20 @@
       <c r="P26" t="n">
         <v>4</v>
       </c>
+      <c r="S26" t="n">
+        <v>21</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Andrew8Kavanagh</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>24.21334</v>
+      </c>
+      <c r="V26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1484,6 +1815,20 @@
       <c r="P27" t="n">
         <v>3</v>
       </c>
+      <c r="S27" t="n">
+        <v>22</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>24.24274</v>
+      </c>
+      <c r="V27" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1530,6 +1875,20 @@
       <c r="P28" t="n">
         <v>3</v>
       </c>
+      <c r="S28" t="n">
+        <v>23</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Dartho Mas</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>24.84136</v>
+      </c>
+      <c r="V28" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1576,6 +1935,22 @@
       <c r="P29" t="n">
         <v>3</v>
       </c>
+      <c r="S29" t="n">
+        <v>24</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1624,6 +1999,22 @@
       <c r="P30" t="n">
         <v>2</v>
       </c>
+      <c r="S30" t="n">
+        <v>24</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>[CSC] OccasionallyAmazingGamer</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1672,6 +2063,22 @@
       <c r="P31" t="n">
         <v>2</v>
       </c>
+      <c r="S31" t="n">
+        <v>24</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>daytime</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1720,6 +2127,20 @@
       <c r="P32" t="n">
         <v>2</v>
       </c>
+      <c r="S32" t="n">
+        <v>27</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>DragonBlood91D</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>24.69515</v>
+      </c>
+      <c r="V32" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1766,6 +2187,20 @@
       <c r="P33" t="n">
         <v>1</v>
       </c>
+      <c r="S33" t="n">
+        <v>28</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Orb Bee Bob</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>25.16888</v>
+      </c>
+      <c r="V33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1814,6 +2249,20 @@
       <c r="P34" t="n">
         <v>1</v>
       </c>
+      <c r="S34" t="n">
+        <v>29</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="U34" t="n">
+        <v>25.45664</v>
+      </c>
+      <c r="V34" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1862,6 +2311,22 @@
       <c r="P35" t="n">
         <v>1</v>
       </c>
+      <c r="S35" t="n">
+        <v>30</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Es3en</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="G36" t="n">
@@ -1878,6 +2343,22 @@
       <c r="J36" t="n">
         <v>1</v>
       </c>
+      <c r="S36" t="n">
+        <v>30</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Gruselda1</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="G37" t="n">
@@ -1894,7 +2375,120 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
-    </row>
+      <c r="S37" t="n">
+        <v>30</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Minixerces2116</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="S38" t="n">
+        <v>30</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Waaksaam</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="S39" t="n">
+        <v>30</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>[20x]K410K3N</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="S40" t="n">
+        <v>30</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>[CSC] redal</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="S41" t="n">
+        <v>30</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>[CSC]ShyGirlyRaccoon</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="S42" t="n">
+        <v>30</v>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>[MIT] nilswa</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Petite Cup 45 (S3 R16): justMaki wins, LKat 3rd
- Maps: Små Äventyr (ZOMAN) + Flicka Da Kist (JakeAdjacent) — both mappers excluded
- Maki extends S3 win streak to 11/15 (perfect S3 podium + top-5 record continues)
- LKat attended as "Jake Replacement's Replacement" — alias added, verified via Steam ID match
- Drops now active in S3 (16/22 played, best 15)
- SOF 88.6%
</commit_message>
<xml_diff>
--- a/Petite Cups 41-45.xlsx
+++ b/Petite Cups 41-45.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:V49"/>
+  <dimension ref="A2:AB42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -437,6 +437,11 @@
           <t>Petite Cup 44</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Petite Cup 45</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -459,6 +464,11 @@
           <t>Maps: PCDJ - Dungeon Descent + PCDJ 44 - Petite Tropiques Féminins</t>
         </is>
       </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Maps: Cup 45 - Sma Aventyr by ZOMAN + Cup 45 - Flicka Da Kist by [SWMG]JakeAdjacent</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,6 +547,26 @@
         </is>
       </c>
       <c r="V5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -587,6 +617,17 @@
       <c r="U6" t="n">
         <v>24.49382</v>
       </c>
+      <c r="Y6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="AA6" t="n">
+        <v>23.76018</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -645,6 +686,20 @@
       <c r="V7" t="n">
         <v>15</v>
       </c>
+      <c r="Y7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>[KURK] Quickracer10</t>
+        </is>
+      </c>
+      <c r="AA7" t="n">
+        <v>23.83924</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -703,6 +758,20 @@
       <c r="V8" t="n">
         <v>14</v>
       </c>
+      <c r="Y8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Jake Replacement's Replacement</t>
+        </is>
+      </c>
+      <c r="AA8" t="n">
+        <v>22.09842</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -763,6 +832,20 @@
       <c r="V9" t="n">
         <v>13</v>
       </c>
+      <c r="Y9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>23.90383</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -821,6 +904,20 @@
       <c r="V10" t="n">
         <v>12</v>
       </c>
+      <c r="Y10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>[TTR]Heart-TGV</t>
+        </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>22.71883</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -881,6 +978,20 @@
       <c r="V11" t="n">
         <v>11</v>
       </c>
+      <c r="Y11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>[CSC]Tommygaming</t>
+        </is>
+      </c>
+      <c r="AA11" t="n">
+        <v>24.45553</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -939,6 +1050,20 @@
       <c r="V12" t="n">
         <v>10</v>
       </c>
+      <c r="Y12" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>[Quac] microways</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>22.53104</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -997,6 +1122,22 @@
       <c r="V13" t="n">
         <v>10</v>
       </c>
+      <c r="Y13" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1055,6 +1196,20 @@
       <c r="V14" t="n">
         <v>9</v>
       </c>
+      <c r="Y14" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>24.1411</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1117,6 +1272,20 @@
       <c r="V15" t="n">
         <v>9</v>
       </c>
+      <c r="Y15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>24.33339</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1175,6 +1344,20 @@
       <c r="V16" t="n">
         <v>8</v>
       </c>
+      <c r="Y16" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="AA16" t="n">
+        <v>23.2908</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1233,6 +1416,20 @@
       <c r="V17" t="n">
         <v>8</v>
       </c>
+      <c r="Y17" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>felix</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>23.47574</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1291,6 +1488,20 @@
       <c r="V18" t="n">
         <v>7</v>
       </c>
+      <c r="Y18" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>24.62024</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1351,6 +1562,20 @@
       <c r="V19" t="n">
         <v>7</v>
       </c>
+      <c r="Y19" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>24.63227</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1411,6 +1636,20 @@
       <c r="V20" t="n">
         <v>6</v>
       </c>
+      <c r="Y20" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>BB_Benji</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>24.63536</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1469,6 +1708,20 @@
       <c r="V21" t="n">
         <v>6</v>
       </c>
+      <c r="Y21" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>25.86275</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1529,6 +1782,20 @@
       <c r="V22" t="n">
         <v>6</v>
       </c>
+      <c r="Y22" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>26.00999</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1587,6 +1854,22 @@
       <c r="V23" t="n">
         <v>5</v>
       </c>
+      <c r="Y23" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>[CSC] redal</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1647,6 +1930,20 @@
       <c r="V24" t="n">
         <v>5</v>
       </c>
+      <c r="Y24" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>M4rv</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>24.70947</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1707,6 +2004,20 @@
       <c r="V25" t="n">
         <v>5</v>
       </c>
+      <c r="Y25" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>penqwin</t>
+        </is>
+      </c>
+      <c r="AA25" t="n">
+        <v>24.77387</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1769,6 +2080,20 @@
       <c r="V26" t="n">
         <v>4</v>
       </c>
+      <c r="Y26" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>[EEN] Hang Chang-Pang</t>
+        </is>
+      </c>
+      <c r="AA26" t="n">
+        <v>24.78214</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1829,6 +2154,20 @@
       <c r="V27" t="n">
         <v>4</v>
       </c>
+      <c r="Y27" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="AA27" t="n">
+        <v>29.7186</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1889,6 +2228,22 @@
       <c r="V28" t="n">
         <v>4</v>
       </c>
+      <c r="Y28" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>[CSC]ShyGirlyRaccoon</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1951,6 +2306,22 @@
       <c r="V29" t="n">
         <v>3</v>
       </c>
+      <c r="Y29" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>wunderBarr</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2015,6 +2386,20 @@
       <c r="V30" t="n">
         <v>3</v>
       </c>
+      <c r="Y30" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Waaksaam</t>
+        </is>
+      </c>
+      <c r="AA30" t="n">
+        <v>25.16173</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2079,6 +2464,20 @@
       <c r="V31" t="n">
         <v>3</v>
       </c>
+      <c r="Y31" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="AA31" t="n">
+        <v>25.1732</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2141,6 +2540,20 @@
       <c r="V32" t="n">
         <v>2</v>
       </c>
+      <c r="Y32" t="n">
+        <v>27</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="AA32" t="n">
+        <v>25.90704</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2201,6 +2614,22 @@
       <c r="V33" t="n">
         <v>2</v>
       </c>
+      <c r="Y33" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Timmer933</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2263,6 +2692,22 @@
       <c r="V34" t="n">
         <v>2</v>
       </c>
+      <c r="Y34" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>grop44</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2327,6 +2772,22 @@
       <c r="V35" t="n">
         <v>1</v>
       </c>
+      <c r="Y35" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>racemaniac</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="36">
       <c r="G36" t="n">
@@ -2359,6 +2820,22 @@
       <c r="V36" t="n">
         <v>1</v>
       </c>
+      <c r="Y36" t="n">
+        <v>31</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="G37" t="n">
@@ -2391,6 +2868,22 @@
       <c r="V37" t="n">
         <v>1</v>
       </c>
+      <c r="Y37" t="n">
+        <v>31</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>huhconduct</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="S38" t="n">
@@ -2482,13 +2975,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>